<commit_message>
Update CTA report Excel with latest Amplitude numbers
Test traffic excluded: 21 impressions, 0 clicks across 8 CTAs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CTA_노출클릭_정리.xlsx
+++ b/CTA_노출클릭_정리.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\choidayoon\OneDrive\바탕 화면\Landing 실습\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DDF0DE-297E-404A-92A0-7C3A129A5B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307FBAA5-AEDA-4A5C-9D0E-65952FEA2448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2130" yWindow="555" windowWidth="24360" windowHeight="14925" xr2:uid="{1D067AC2-27EF-4690-A09F-ABBE9EE3C1B3}"/>
   </bookViews>
@@ -27,14 +27,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="83">
   <si>
     <t>한입배달 랜딩페이지 CTA별 노출·클릭 현황</t>
   </si>
   <si>
-    <t>기간: 최근 30일 (2026-09-26 ~ 2026-10-26, 조회 2026-10-26)  ·  출처: Amplitude 프로젝트 887090  ·  기준과 제외 조건은 '기준·출처' 시트 참고</t>
-  </si>
-  <si>
     <t>CTA 정보</t>
   </si>
   <si>
@@ -152,9 +149,6 @@
     <t>※ 노출·클릭 수는 Amplitude에서 조회한 값(직접 입력), 클릭률·합계는 수식입니다. 노출은 페이지뷰당 CTA별 1회, 클릭은 누를 때마다 기록되어 클릭 수가 노출 수보다 클 수도 있습니다.</t>
   </si>
   <si>
-    <t>※ 2026-10-26 현재 실제 데이터는 UTM 없이 들어온 방문 1회뿐이라(첫 화면의 topbar·hero만 노출, 클릭 없음) CTA 간 클릭률 비교는 아직 의미가 없습니다.</t>
-  </si>
-  <si>
     <t>노출 / 클릭 이벤트 정의</t>
   </si>
   <si>
@@ -267,6 +261,23 @@
   </si>
   <si>
     <t>https://app.amplitude.com/analytics/orange-water-758048/dashboard/nahopd9w</t>
+  </si>
+  <si>
+    <t>기간: 최근 30일 (2026-09-26 ~ 2026-10-26, 데이터는 모두 10-26) · 조회 2026-10-26 분석 보고서 작성 후 재조회 · 출처: Amplitude 프로젝트 887090 · 기준은 '기준·출처' 시트 참고</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>※ 2026-10-26 현재 테스트를 뺀 방문자는 7명(자동화 브라우저 1명 포함), CTA 노출 21회, 클릭 0회입니다. 표본이 작아 CTA 간 클릭률 비교는 아직 의미가 없습니다(버튼별 노출 100회 이후 비교 권장).</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-10-26 (분석 보고서 작성 후 재조회, Amplitude 캐시를 피하려고 조회 범위를 최근 14일로 바꿔 확인 · 데이터는 모두 10-26)</t>
+  </si>
+  <si>
+    <t>분석 보고서</t>
+  </si>
+  <si>
+    <t>https://claude.ai/artifact/PMPdDzeyqwEUBT4mhBpyGE</t>
   </si>
 </sst>
 </file>
@@ -1308,61 +1319,61 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>1</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="31" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="31"/>
       <c r="C3" s="31"/>
       <c r="D3" s="31"/>
       <c r="E3" s="31"/>
       <c r="F3" s="32" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G3" s="32"/>
       <c r="H3" s="32"/>
       <c r="I3" s="33" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J3" s="33"/>
       <c r="K3" s="33"/>
     </row>
     <row r="4" spans="1:11" ht="45.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="G4" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="29" t="s">
+      <c r="H4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="30" t="s">
+      <c r="J4" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="30" t="s">
+      <c r="K4" s="30" t="s">
         <v>14</v>
-      </c>
-      <c r="K4" s="30" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="90.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1371,16 +1382,16 @@
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>18</v>
-      </c>
       <c r="F5" s="10">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G5" s="11">
         <v>0</v>
@@ -1390,14 +1401,14 @@
         <v>0</v>
       </c>
       <c r="I5" s="13">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J5" s="13">
         <v>1</v>
       </c>
       <c r="K5" s="14">
         <f t="shared" ref="K5:K13" si="1">IF(I5=0,"-",J5/I5)</f>
-        <v>0.5</v>
+        <v>0.14285714285714285</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="117.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1406,16 +1417,16 @@
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>21</v>
-      </c>
       <c r="F6" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G6" s="11">
         <v>0</v>
@@ -1425,14 +1436,14 @@
         <v>0</v>
       </c>
       <c r="I6" s="13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J6" s="13">
         <v>1</v>
       </c>
       <c r="K6" s="14">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="117.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1441,26 +1452,26 @@
       </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E7" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>24</v>
-      </c>
       <c r="F7" s="10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G7" s="11">
         <v>0</v>
       </c>
-      <c r="H7" s="12" t="str">
+      <c r="H7" s="12">
         <f t="shared" si="0"/>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="I7" s="13">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J7" s="13">
         <v>0</v>
@@ -1476,26 +1487,26 @@
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="E8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="9" t="s">
-        <v>27</v>
-      </c>
       <c r="F8" s="10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8" s="11">
         <v>0</v>
       </c>
-      <c r="H8" s="12" t="str">
+      <c r="H8" s="12">
         <f t="shared" si="0"/>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="I8" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J8" s="13">
         <v>0</v>
@@ -1511,26 +1522,26 @@
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="E9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="9" t="s">
-        <v>30</v>
-      </c>
       <c r="F9" s="10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="11">
         <v>0</v>
       </c>
-      <c r="H9" s="12" t="str">
+      <c r="H9" s="12">
         <f t="shared" si="0"/>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="I9" s="13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="13">
         <v>0</v>
@@ -1546,26 +1557,26 @@
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="E10" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>33</v>
-      </c>
       <c r="F10" s="10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10" s="11">
         <v>0</v>
       </c>
-      <c r="H10" s="12" t="str">
+      <c r="H10" s="12">
         <f t="shared" si="0"/>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="I10" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J10" s="13">
         <v>0</v>
@@ -1581,26 +1592,26 @@
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>35</v>
-      </c>
       <c r="E11" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F11" s="10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G11" s="11">
         <v>0</v>
       </c>
-      <c r="H11" s="12" t="str">
+      <c r="H11" s="12">
         <f t="shared" si="0"/>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="I11" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11" s="13">
         <v>0</v>
@@ -1616,26 +1627,26 @@
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="E12" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="9" t="s">
-        <v>38</v>
-      </c>
       <c r="F12" s="10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G12" s="11">
         <v>0</v>
       </c>
-      <c r="H12" s="12" t="str">
+      <c r="H12" s="12">
         <f t="shared" si="0"/>
-        <v>-</v>
+        <v>0</v>
       </c>
       <c r="I12" s="13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J12" s="13">
         <v>0</v>
@@ -1649,13 +1660,13 @@
       <c r="A13" s="15"/>
       <c r="B13" s="16"/>
       <c r="C13" s="16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D13" s="17"/>
       <c r="E13" s="17"/>
       <c r="F13" s="18">
         <f>SUM(F5:F12)</f>
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="G13" s="18">
         <f>SUM(G5:G12)</f>
@@ -1667,7 +1678,7 @@
       </c>
       <c r="I13" s="20">
         <f>SUM(I5:I12)</f>
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="J13" s="20">
         <f>SUM(J5:J12)</f>
@@ -1675,17 +1686,17 @@
       </c>
       <c r="K13" s="21">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>6.8965517241379309E-2</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1716,72 +1727,72 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="D3" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="E3" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="F3" s="22" t="s">
         <v>46</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="F3" s="22" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="27" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>52</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="D5" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="E5" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="F5" s="9" t="s">
         <v>58</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1792,7 +1803,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E645A9B7-C4BE-4AFD-97EC-C86737155F86}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.625" style="1" customWidth="1"/>
@@ -1802,79 +1813,87 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="25" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="B5" s="26">
-        <v>46321</v>
+        <v>65</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B10" s="27" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B11" s="27" t="s">
-        <v>79</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A12" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="27" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1882,6 +1901,7 @@
   <hyperlinks>
     <hyperlink ref="B10" r:id="rId1" xr:uid="{AE849670-B6DF-4867-BFF4-7A0F8F988F10}"/>
     <hyperlink ref="B11" r:id="rId2" xr:uid="{4524571B-255B-474F-8ABD-EA6A9094866D}"/>
+    <hyperlink ref="B12" r:id="rId3" xr:uid="{517EBC84-97EA-4E49-B96A-88FD2915C543}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>